<commit_message>
demo: update demo forms
</commit_message>
<xml_diff>
--- a/Demo/ONCHO/ento/river prospection/demo_oncho_priv_prosp_9999_1_river_assess.xlsx
+++ b/Demo/ONCHO/ento/river prospection/demo_oncho_priv_prosp_9999_1_river_assess.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\ONCHO\ento\river prospection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68FFD7E3-0EA6-462A-852A-BF2C2C26A01F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A473C95-271D-4414-93A1-D51D55BF3956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1533" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="316">
   <si>
     <t>type</t>
   </si>
@@ -977,6 +977,12 @@
   </si>
   <si>
     <t>More than 201</t>
+  </si>
+  <si>
+    <t>${s_site_suitability} = 'Yes'</t>
+  </si>
+  <si>
+    <t>${s_larvae_evidence} = 'Yes'</t>
   </si>
 </sst>
 </file>
@@ -1988,7 +1994,9 @@
       <c r="E20" s="21"/>
       <c r="F20" s="21"/>
       <c r="G20" s="23"/>
-      <c r="H20" s="22"/>
+      <c r="H20" s="22" t="s">
+        <v>314</v>
+      </c>
       <c r="I20" s="22"/>
       <c r="J20" s="22" t="s">
         <v>11</v>
@@ -2011,7 +2019,9 @@
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="23"/>
-      <c r="H21" s="22"/>
+      <c r="H21" s="22" t="s">
+        <v>315</v>
+      </c>
       <c r="I21" s="22"/>
       <c r="J21" s="22" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
demo: update oncho forms
</commit_message>
<xml_diff>
--- a/Demo/ONCHO/ento/river prospection/demo_oncho_priv_prosp_9999_1_river_assess.xlsx
+++ b/Demo/ONCHO/ento/river prospection/demo_oncho_priv_prosp_9999_1_river_assess.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\ONCHO\ento\river prospection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A473C95-271D-4414-93A1-D51D55BF3956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D9DA7F-BB08-456A-91ED-CF37DAA988E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1539" uniqueCount="318">
   <si>
     <t>type</t>
   </si>
@@ -983,6 +983,12 @@
   </si>
   <si>
     <t>${s_larvae_evidence} = 'Yes'</t>
+  </si>
+  <si>
+    <t>s_river_basin</t>
+  </si>
+  <si>
+    <t>River Basin</t>
   </si>
 </sst>
 </file>
@@ -1477,7 +1483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="26" style="3" customWidth="1"/>
@@ -1811,15 +1817,15 @@
       <c r="L12" s="21"/>
       <c r="M12" s="21"/>
     </row>
-    <row r="13" spans="1:13" s="4" customFormat="1" ht="31.5">
+    <row r="13" spans="1:13" s="4" customFormat="1">
       <c r="A13" s="21" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>21</v>
+        <v>316</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>101</v>
+        <v>317</v>
       </c>
       <c r="D13" s="23"/>
       <c r="E13" s="21"/>
@@ -1834,70 +1840,66 @@
       <c r="L13" s="21"/>
       <c r="M13" s="21"/>
     </row>
-    <row r="14" spans="1:13" s="4" customFormat="1">
+    <row r="14" spans="1:13" s="4" customFormat="1" ht="31.5">
       <c r="A14" s="21" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D14" s="23"/>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
       <c r="J14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="K14" s="21"/>
+      <c r="K14" s="22"/>
       <c r="L14" s="21"/>
       <c r="M14" s="21"/>
     </row>
     <row r="15" spans="1:13" s="4" customFormat="1">
       <c r="A15" s="21" t="s">
-        <v>289</v>
+        <v>22</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>283</v>
+        <v>23</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>287</v>
+        <v>102</v>
       </c>
       <c r="D15" s="23"/>
       <c r="E15" s="21"/>
       <c r="F15" s="21"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="21"/>
       <c r="J15" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="K15" s="22"/>
+      <c r="K15" s="21"/>
       <c r="L15" s="21"/>
       <c r="M15" s="21"/>
     </row>
     <row r="16" spans="1:13" s="4" customFormat="1">
       <c r="A16" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D16" s="23"/>
       <c r="E16" s="21"/>
-      <c r="F16" s="21" t="s">
-        <v>291</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>292</v>
-      </c>
+      <c r="F16" s="21"/>
+      <c r="G16" s="23"/>
       <c r="H16" s="22"/>
       <c r="I16" s="22"/>
       <c r="J16" s="22" t="s">
@@ -1909,21 +1911,21 @@
     </row>
     <row r="17" spans="1:13" s="4" customFormat="1">
       <c r="A17" s="21" t="s">
-        <v>9</v>
+        <v>290</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D17" s="23"/>
       <c r="E17" s="21"/>
       <c r="F17" s="21" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="H17" s="22"/>
       <c r="I17" s="22"/>
@@ -1936,18 +1938,22 @@
     </row>
     <row r="18" spans="1:13" s="4" customFormat="1">
       <c r="A18" s="21" t="s">
-        <v>297</v>
+        <v>9</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="23"/>
+      <c r="F18" s="21" t="s">
+        <v>293</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>294</v>
+      </c>
       <c r="H18" s="22"/>
       <c r="I18" s="22"/>
       <c r="J18" s="22" t="s">
@@ -1957,15 +1963,15 @@
       <c r="L18" s="21"/>
       <c r="M18" s="21"/>
     </row>
-    <row r="19" spans="1:13" s="4" customFormat="1" ht="31.5">
+    <row r="19" spans="1:13" s="4" customFormat="1">
       <c r="A19" s="21" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D19" s="23"/>
       <c r="E19" s="21"/>
@@ -1985,18 +1991,16 @@
         <v>305</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D20" s="23"/>
       <c r="E20" s="21"/>
       <c r="F20" s="21"/>
       <c r="G20" s="23"/>
-      <c r="H20" s="22" t="s">
-        <v>314</v>
-      </c>
+      <c r="H20" s="22"/>
       <c r="I20" s="22"/>
       <c r="J20" s="22" t="s">
         <v>11</v>
@@ -2006,21 +2010,21 @@
       <c r="M20" s="21"/>
     </row>
     <row r="21" spans="1:13" s="4" customFormat="1" ht="31.5">
-      <c r="A21" s="32" t="s">
-        <v>306</v>
+      <c r="A21" s="21" t="s">
+        <v>305</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D21" s="23"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
       <c r="G21" s="23"/>
       <c r="H21" s="22" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I21" s="22"/>
       <c r="J21" s="22" t="s">
@@ -2030,42 +2034,44 @@
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
     </row>
-    <row r="22" spans="1:13">
-      <c r="A22" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="D22" s="27" t="s">
-        <v>269</v>
-      </c>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="21" t="s">
+    <row r="22" spans="1:13" s="4" customFormat="1" ht="31.5">
+      <c r="A22" s="32" t="s">
+        <v>306</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>304</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="D22" s="23"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="22" t="s">
+        <v>315</v>
+      </c>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="K22" s="26"/>
-      <c r="L22" s="26"/>
-      <c r="M22" s="26"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="D23" s="27"/>
+        <v>103</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>269</v>
+      </c>
       <c r="E23" s="26"/>
       <c r="F23" s="26"/>
       <c r="G23" s="27"/>
@@ -2080,13 +2086,13 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="26" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D24" s="27"/>
       <c r="E24" s="26"/>
@@ -2103,13 +2109,13 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="26" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D25" s="27"/>
       <c r="E25" s="26"/>
@@ -2117,20 +2123,22 @@
       <c r="G25" s="27"/>
       <c r="H25" s="26"/>
       <c r="I25" s="26"/>
-      <c r="J25" s="21"/>
+      <c r="J25" s="21" t="s">
+        <v>11</v>
+      </c>
       <c r="K25" s="26"/>
       <c r="L25" s="26"/>
       <c r="M25" s="26"/>
     </row>
     <row r="26" spans="1:13">
       <c r="A26" s="26" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D26" s="27"/>
       <c r="E26" s="26"/>
@@ -2145,13 +2153,13 @@
     </row>
     <row r="27" spans="1:13">
       <c r="A27" s="26" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D27" s="27"/>
       <c r="E27" s="26"/>
@@ -2166,21 +2174,19 @@
     </row>
     <row r="28" spans="1:13">
       <c r="A28" s="26" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D28" s="27"/>
       <c r="E28" s="26"/>
       <c r="F28" s="26"/>
       <c r="G28" s="27"/>
-      <c r="H28" s="26" t="s">
-        <v>34</v>
-      </c>
+      <c r="H28" s="26"/>
       <c r="I28" s="26"/>
       <c r="J28" s="21"/>
       <c r="K28" s="26"/>
@@ -2189,67 +2195,67 @@
     </row>
     <row r="29" spans="1:13">
       <c r="A29" s="26" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>270</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="D29" s="27"/>
       <c r="E29" s="26"/>
       <c r="F29" s="26"/>
       <c r="G29" s="27"/>
-      <c r="H29" s="26"/>
+      <c r="H29" s="26" t="s">
+        <v>34</v>
+      </c>
       <c r="I29" s="26"/>
-      <c r="J29" s="21" t="s">
-        <v>11</v>
-      </c>
+      <c r="J29" s="21"/>
       <c r="K29" s="26"/>
       <c r="L29" s="26"/>
       <c r="M29" s="26"/>
     </row>
-    <row r="30" spans="1:13" s="4" customFormat="1">
-      <c r="A30" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="D30" s="23"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
+    <row r="30" spans="1:13">
+      <c r="A30" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
     </row>
     <row r="31" spans="1:13" s="4" customFormat="1">
       <c r="A31" s="21" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D31" s="23"/>
       <c r="E31" s="21"/>
       <c r="F31" s="21"/>
       <c r="G31" s="24"/>
-      <c r="H31" s="26" t="s">
-        <v>40</v>
-      </c>
+      <c r="H31" s="21"/>
       <c r="I31" s="21"/>
       <c r="J31" s="22"/>
       <c r="K31" s="21"/>
@@ -2258,17 +2264,21 @@
     </row>
     <row r="32" spans="1:13" s="4" customFormat="1">
       <c r="A32" s="21" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="23"/>
+        <v>39</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>112</v>
+      </c>
       <c r="D32" s="23"/>
       <c r="E32" s="21"/>
       <c r="F32" s="21"/>
       <c r="G32" s="24"/>
-      <c r="H32" s="21"/>
+      <c r="H32" s="26" t="s">
+        <v>40</v>
+      </c>
       <c r="I32" s="21"/>
       <c r="J32" s="22"/>
       <c r="K32" s="21"/>
@@ -2277,10 +2287,10 @@
     </row>
     <row r="33" spans="1:13" s="4" customFormat="1">
       <c r="A33" s="21" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C33" s="23"/>
       <c r="D33" s="23"/>
@@ -2295,9 +2305,23 @@
       <c r="M33" s="21"/>
     </row>
     <row r="34" spans="1:13" s="4" customFormat="1">
-      <c r="B34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="G34" s="3"/>
+      <c r="A34" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+      <c r="M34" s="21"/>
     </row>
     <row r="35" spans="1:13" s="4" customFormat="1">
       <c r="B35" s="7"/>
@@ -2305,9 +2329,14 @@
       <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:13" s="4" customFormat="1">
-      <c r="B36" s="3"/>
-      <c r="D36" s="3"/>
+      <c r="B36" s="7"/>
+      <c r="D36" s="7"/>
       <c r="G36" s="3"/>
+    </row>
+    <row r="37" spans="1:13" s="4" customFormat="1">
+      <c r="B37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="G37" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>